<commit_message>
Add day-unit cover rules, coordinator-only leave authorisation, hosting and security plan
Also: generator now shows leavers as Not in post and checks the RGH/NHH day units.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8EjimpErkij9gvKaTvnbV
</commit_message>
<xml_diff>
--- a/docs/samples/haematology-roster-export-sample.xlsx
+++ b/docs/samples/haematology-roster-export-sample.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About this file" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Residents &amp; Registrars'!$A$1:$R$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Residents &amp; Registrars'!$A$1:$S$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +50,11 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <sz val="9"/>
     </font>
     <font>
@@ -65,7 +70,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -79,7 +84,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007030A0"/>
+        <fgColor rgb="00C00000"/>
       </patternFill>
     </fill>
     <fill>
@@ -90,6 +95,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="006FB1EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00595959"/>
       </patternFill>
     </fill>
     <fill>
@@ -114,12 +124,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00262626"/>
+        <fgColor rgb="007030A0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
+        <fgColor rgb="00262626"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -172,46 +182,49 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -577,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -596,8 +609,9 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -635,72 +649,78 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>F2 (left 06/11)
+J. Reid</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>F2 (on calls NHH)
 T. Hughes</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>IMT2
 S. Malik</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>IMT3
 B. Carter</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>JCF
 L. Osei</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Registrar
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Middle grade
 Omar</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Registrar
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Middle grade
 Hannah</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Registrar
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Middle grade
 Daniel</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Registrar
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Middle grade
 Zara</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Registrar
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Middle grade
 Meera</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Registrar
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Middle grade
 Yusuf</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Resident cover</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Registrar cover</t>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Middle grade / day units</t>
         </is>
       </c>
     </row>
@@ -720,7 +740,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>AVOID</t>
+          <t>NO AL</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -735,62 +755,67 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
           <t>TWILIGHT</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
           <t>GUH</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>GUH LAB</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>RGH - DAY UNIT</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>GUH LAB</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>RGH MDCU</t>
         </is>
       </c>
-      <c r="Q2" s="8" t="inlineStr">
+      <c r="R2" s="8" t="inlineStr">
         <is>
           <t>GUH OK · RGH OK · NHH n/a</t>
         </is>
       </c>
-      <c r="R2" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
+      <c r="S2" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU closed</t>
         </is>
       </c>
     </row>
@@ -810,7 +835,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>AVOID</t>
+          <t>NO AL</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -818,160 +843,170 @@
           <t>GUH</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>NHH</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
           <t>TWILIGHT</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>GUH LAB</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>NHH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="M3" s="7" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>GUH LAB</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="R3" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH OK · NHH OK</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="10" t="n">
+        <v>46344</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Dr Fraser</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>NHH</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>STUDY LEAVE</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>GUH LAB</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="Q3" s="8" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="M4" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>NHH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
         <is>
           <t>GUH OK · RGH OK · NHH OK</t>
         </is>
       </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="n">
-        <v>46344</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Dr Fraser</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>STUDY LEAVE</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="L4" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="M4" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="Q4" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-      <c r="R4" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU OK</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="10" t="n">
         <v>46345</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -990,722 +1025,777 @@
           <t>GUH</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>NHH</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
           <t>TWILIGHT</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>RGH DAY UNIT</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>LONG DAY</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="L5" s="11" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="M5" s="12" t="inlineStr">
         <is>
           <t>ANNUAL LEAVE</t>
         </is>
       </c>
-      <c r="M5" s="7" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>NHH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH OK · NHH OK</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="13" t="n">
+        <v>46346</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Dr Fraser</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>NIGHTS</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>LONG DAY</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="M6" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>NHH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="P6" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="R6" s="14" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH OK · NHH GAP</t>
+        </is>
+      </c>
+      <c r="S6" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="n">
+        <v>46347</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>NIGHTS</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>LONG DAY</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="n"/>
+      <c r="M7" s="17" t="n"/>
+      <c r="N7" s="17" t="n"/>
+      <c r="O7" s="17" t="n"/>
+      <c r="P7" s="17" t="n"/>
+      <c r="Q7" s="17" t="n"/>
+      <c r="R7" s="18" t="n"/>
+      <c r="S7" s="18" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="15" t="n">
+        <v>46348</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n"/>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>NIGHTS</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
+      <c r="J8" s="17" t="n"/>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>LONG DAY</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="n"/>
+      <c r="M8" s="17" t="n"/>
+      <c r="N8" s="17" t="n"/>
+      <c r="O8" s="17" t="n"/>
+      <c r="P8" s="17" t="n"/>
+      <c r="Q8" s="17" t="n"/>
+      <c r="R8" s="18" t="n"/>
+      <c r="S8" s="18" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="10" t="n">
+        <v>46349</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Dr Lin</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="N9" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>GUH LAB</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH OK · NHH n/a</t>
+        </is>
+      </c>
+      <c r="S9" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="10" t="n">
+        <v>46350</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Dr Lin</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
         <is>
           <t>NHH</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>NHH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>RGH MDCU</t>
+        </is>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH OK · NHH OK</t>
+        </is>
+      </c>
+      <c r="S10" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="10" t="n">
+        <v>46351</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Dr Lin</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>NHH</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>WARD COVER</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="P5" s="5" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>NHH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="P11" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
         <is>
           <t>RGH</t>
         </is>
       </c>
-      <c r="Q5" s="8" t="inlineStr">
+      <c r="R11" s="8" t="inlineStr">
         <is>
           <t>GUH OK · RGH OK · NHH OK</t>
         </is>
       </c>
-      <c r="R5" s="8" t="inlineStr">
+      <c r="S11" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="10" t="n">
+        <v>46352</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Dr Lin</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>NHH</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>RGH AM; PM ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="M12" s="12" t="inlineStr">
+        <is>
+          <t>SpR TRAINING DAY</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>NHH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="P12" s="19" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE (PENDING)</t>
+        </is>
+      </c>
+      <c r="Q12" s="11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
         <is>
           <t>GUH OK · RGH OK · NHH OK</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="n">
-        <v>46346</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="S12" s="14" t="inlineStr">
+        <is>
+          <t>GUH AT RISK (leave requested) · RGH DU OK · NHH DU OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="10" t="n">
+        <v>46353</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Dr Fraser</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>NIGHTS</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Dr Lin</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>NHH</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>OFF PRE ON-CALL</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>RGH</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>RGH - DAY UNIT</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="N13" s="11" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="O13" s="12" t="inlineStr">
+        <is>
+          <t>ANNUAL LEAVE</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>GUH</t>
+        </is>
+      </c>
+      <c r="Q13" s="12" t="inlineStr">
+        <is>
+          <t>SICK LEAVE</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH OK · NHH OK</t>
+        </is>
+      </c>
+      <c r="S13" s="8" t="inlineStr">
+        <is>
+          <t>GUH OK · RGH DU OK · NHH DU resident only</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="15" t="n">
+        <v>46354</v>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>LONG DAY</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="L6" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="M6" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="O6" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="P6" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="Q6" s="12" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH GAP</t>
-        </is>
-      </c>
-      <c r="R6" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="n">
-        <v>46347</v>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="14" t="n"/>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>NIGHTS</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="n"/>
-      <c r="H7" s="15" t="n"/>
-      <c r="I7" s="15" t="n"/>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="I14" s="17" t="n"/>
+      <c r="J14" s="17" t="n"/>
+      <c r="K14" s="17" t="n"/>
+      <c r="L14" s="17" t="n"/>
+      <c r="M14" s="17" t="n"/>
+      <c r="N14" s="17" t="n"/>
+      <c r="O14" s="17" t="n"/>
+      <c r="P14" s="17" t="n"/>
+      <c r="Q14" s="17" t="n"/>
+      <c r="R14" s="18" t="n"/>
+      <c r="S14" s="18" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="n">
+        <v>46355</v>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>NOT IN POST</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>LONG DAY</t>
         </is>
       </c>
-      <c r="K7" s="15" t="n"/>
-      <c r="L7" s="15" t="n"/>
-      <c r="M7" s="15" t="n"/>
-      <c r="N7" s="15" t="n"/>
-      <c r="O7" s="15" t="n"/>
-      <c r="P7" s="15" t="n"/>
-      <c r="Q7" s="16" t="n"/>
-      <c r="R7" s="16" t="n"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="13" t="n">
-        <v>46348</v>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>NIGHTS</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="n"/>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="15" t="n"/>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>LONG DAY</t>
-        </is>
-      </c>
-      <c r="K8" s="15" t="n"/>
-      <c r="L8" s="15" t="n"/>
-      <c r="M8" s="15" t="n"/>
-      <c r="N8" s="15" t="n"/>
-      <c r="O8" s="15" t="n"/>
-      <c r="P8" s="15" t="n"/>
-      <c r="Q8" s="16" t="n"/>
-      <c r="R8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="17" t="n">
-        <v>46349</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Dr Lin</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>NO AL</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="M9" s="7" t="inlineStr">
-        <is>
-          <t>NHH - DAY UNIT</t>
-        </is>
-      </c>
-      <c r="N9" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>GUH LAB</t>
-        </is>
-      </c>
-      <c r="P9" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="Q9" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH n/a</t>
-        </is>
-      </c>
-      <c r="R9" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="9" t="n">
-        <v>46350</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Dr Lin</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="M10" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="N10" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="P10" s="5" t="inlineStr">
-        <is>
-          <t>RGH MDCU</t>
-        </is>
-      </c>
-      <c r="Q10" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-      <c r="R10" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="9" t="n">
-        <v>46351</v>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Dr Lin</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>WARD COVER</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="M11" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="N11" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="O11" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="P11" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="Q11" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-      <c r="R11" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="9" t="n">
-        <v>46352</v>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Dr Lin</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>RGH AM; PM ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="L12" s="11" t="inlineStr">
-        <is>
-          <t>SpR TRAINING DAY</t>
-        </is>
-      </c>
-      <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="N12" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="O12" s="18" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE (PENDING)</t>
-        </is>
-      </c>
-      <c r="P12" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="Q12" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-      <c r="R12" s="12" t="inlineStr">
-        <is>
-          <t>GUH AT RISK (pending leave) · RGH OK · NHH OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="9" t="n">
-        <v>46353</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Dr Lin</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>NHH</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>OFF PRE ON-CALL</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>RGH</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="M13" s="10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="N13" s="11" t="inlineStr">
-        <is>
-          <t>ANNUAL LEAVE</t>
-        </is>
-      </c>
-      <c r="O13" s="4" t="inlineStr">
-        <is>
-          <t>GUH</t>
-        </is>
-      </c>
-      <c r="P13" s="11" t="inlineStr">
-        <is>
-          <t>SICK LEAVE</t>
-        </is>
-      </c>
-      <c r="Q13" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH OK</t>
-        </is>
-      </c>
-      <c r="R13" s="8" t="inlineStr">
-        <is>
-          <t>GUH OK · RGH OK · NHH none (ideal only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="13" t="n">
-        <v>46354</v>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n"/>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>LONG DAY</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="n"/>
-      <c r="I14" s="15" t="n"/>
-      <c r="J14" s="15" t="n"/>
-      <c r="K14" s="15" t="n"/>
-      <c r="L14" s="15" t="n"/>
-      <c r="M14" s="15" t="n"/>
-      <c r="N14" s="15" t="n"/>
-      <c r="O14" s="15" t="n"/>
-      <c r="P14" s="15" t="n"/>
-      <c r="Q14" s="16" t="n"/>
-      <c r="R14" s="16" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="13" t="n">
-        <v>46355</v>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>LONG DAY</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="n"/>
-      <c r="I15" s="15" t="n"/>
-      <c r="J15" s="15" t="n"/>
-      <c r="K15" s="15" t="n"/>
-      <c r="L15" s="15" t="n"/>
-      <c r="M15" s="15" t="n"/>
-      <c r="N15" s="15" t="n"/>
-      <c r="O15" s="15" t="n"/>
-      <c r="P15" s="15" t="n"/>
-      <c r="Q15" s="16" t="n"/>
-      <c r="R15" s="16" t="n"/>
+      <c r="I15" s="17" t="n"/>
+      <c r="J15" s="17" t="n"/>
+      <c r="K15" s="17" t="n"/>
+      <c r="L15" s="17" t="n"/>
+      <c r="M15" s="17" t="n"/>
+      <c r="N15" s="17" t="n"/>
+      <c r="O15" s="17" t="n"/>
+      <c r="P15" s="17" t="n"/>
+      <c r="Q15" s="17" t="n"/>
+      <c r="R15" s="18" t="n"/>
+      <c r="S15" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R15"/>
+  <autoFilter ref="A1:S15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1737,77 +1827,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Request ID</t>
         </is>
       </c>
-      <c r="B1" s="19" t="inlineStr">
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>Submitted</t>
         </is>
       </c>
-      <c r="C1" s="19" t="inlineStr">
+      <c r="C1" s="20" t="inlineStr">
         <is>
           <t>Doctor</t>
         </is>
       </c>
-      <c r="D1" s="19" t="inlineStr">
+      <c r="D1" s="20" t="inlineStr">
         <is>
           <t>Grade</t>
         </is>
       </c>
-      <c r="E1" s="19" t="inlineStr">
+      <c r="E1" s="20" t="inlineStr">
         <is>
           <t>Leave type</t>
         </is>
       </c>
-      <c r="F1" s="19" t="inlineStr">
+      <c r="F1" s="20" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="G1" s="19" t="inlineStr">
+      <c r="G1" s="20" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="H1" s="19" t="inlineStr">
+      <c r="H1" s="20" t="inlineStr">
         <is>
           <t>Part of day</t>
         </is>
       </c>
-      <c r="I1" s="19" t="inlineStr">
+      <c r="I1" s="20" t="inlineStr">
         <is>
           <t>Working days</t>
         </is>
       </c>
-      <c r="J1" s="19" t="inlineStr">
+      <c r="J1" s="20" t="inlineStr">
         <is>
           <t>AL remaining after</t>
         </is>
       </c>
-      <c r="K1" s="19" t="inlineStr">
+      <c r="K1" s="20" t="inlineStr">
         <is>
           <t>Proposed cover</t>
         </is>
       </c>
-      <c r="L1" s="19" t="inlineStr">
+      <c r="L1" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="M1" s="19" t="inlineStr">
+      <c r="M1" s="20" t="inlineStr">
         <is>
           <t>Decided by</t>
         </is>
       </c>
-      <c r="N1" s="19" t="inlineStr">
+      <c r="N1" s="20" t="inlineStr">
         <is>
           <t>Decided at</t>
         </is>
       </c>
-      <c r="O1" s="19" t="inlineStr">
+      <c r="O1" s="20" t="inlineStr">
         <is>
           <t>Reason / notes</t>
         </is>

</xml_diff>